<commit_message>
feat: Standardized JSON profiles, integrated BMSA/BMSB to MP-03, and compiled signal pool
</commit_message>
<xml_diff>
--- a/exports/measuring-profiles/MP-03.xlsx
+++ b/exports/measuring-profiles/MP-03.xlsx
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -799,7 +799,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>System/CANBusSystem/cBMSA/SOH</t>
         </is>
       </c>
       <c r="E6" s="10" t="n">
@@ -823,7 +823,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>no present</t>
+          <t>present</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>System/CANBusSystem/cBMSA/TtlDschrgEnergy</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
@@ -869,7 +869,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>no present</t>
+          <t>present</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>System/CANBusSystem/cBMSA/TtlChrgEnergy</t>
         </is>
       </c>
       <c r="E8" s="10" t="n">
@@ -915,7 +915,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>no present</t>
+          <t>present</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>System/CANBusSystem/cBMSA/MaxTemp</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
@@ -961,7 +961,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>no present</t>
+          <t>present</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>System/CANBusSystem/cBMSA/MinTemp</t>
         </is>
       </c>
       <c r="E10" s="10" t="n">
@@ -1003,7 +1003,7 @@
       <c r="I10" s="9" t="n"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>no present</t>
+          <t>present</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>System/CANBusSystem/cBMSA/FaultCode</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>no present</t>
+          <t>present</t>
         </is>
       </c>
     </row>
@@ -1238,46 +1238,414 @@
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>bmsa_voltage</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack A terminal voltage</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSA/Voltage</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>250 ms</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>High speed Pack A voltage; PERF-008</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>bmsa_current</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack A current (signed, +disch / -regen)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSA/Current</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>-800</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>250 ms</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>High speed Pack A current; PERF-008</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>bmsa_soc</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack A state of charge</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSA/SOC</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>1 s</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Pack A energy level; LOAD-010</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>bmsa_temp_max</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack A maximum cell temperature</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSA/MaxTemp</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>5 s</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Pack A thermal monitoring</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>bmsb_voltage</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack B terminal voltage</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSB/Voltage</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>250 ms</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>High speed Pack B voltage; PERF-008</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>bmsb_current</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack B current (signed, +disch / -regen)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSB/Current</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>-800</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>250 ms</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>High speed Pack B current; PERF-008</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>bmsb_soc</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack B state of charge</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSB/SOC</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>1 s</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Pack B energy level; LOAD-010</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>bmsb_temp_max</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack B maximum cell temperature</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSB/MaxTemp</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>5 s</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Pack B thermal monitoring</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>ambient_temp</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Ambient temperature</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E24" s="10" t="n">
         <v>-20</v>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="F24" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G24" s="13" t="inlineStr">
         <is>
           <t>1 min</t>
         </is>
       </c>
-      <c r="H16" s="11" t="n">
+      <c r="H24" s="11" t="n">
         <v>0.0167</v>
       </c>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="I24" s="9" t="inlineStr">
         <is>
           <t>Normalise performance results</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>manual-only</t>
         </is>

</xml_diff>

<commit_message>
feat: Integrated BMSA and BMSB SOH telemetry to MP-03 and updated signal pool
</commit_message>
<xml_diff>
--- a/exports/measuring-profiles/MP-03.xlsx
+++ b/exports/measuring-profiles/MP-03.xlsx
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1424,41 +1424,41 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>bmsb_voltage</t>
+          <t>bmsa_soh</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Battery Pack B terminal voltage</t>
+          <t>Battery Pack A State of Health</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>System/CANBusSystem/cBMSB/Voltage</t>
+          <t>System/CANBusSystem/cBMSA/SOH</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>250 ms</t>
+          <t>1 day</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>4</v>
+        <v>1.16e-05</v>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>High speed Pack B voltage; PERF-008</t>
+          <t>Metric1d</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1470,29 +1470,29 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>bmsb_current</t>
+          <t>bmsb_voltage</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Battery Pack B current (signed, +disch / -regen)</t>
+          <t>Battery Pack B terminal voltage</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>System/CANBusSystem/cBMSB/Current</t>
+          <t>System/CANBusSystem/cBMSB/Voltage</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-800</v>
+        <v>0</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>High speed Pack B current; PERF-008</t>
+          <t>High speed Pack B voltage; PERF-008</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1516,41 +1516,41 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>bmsb_soc</t>
+          <t>bmsb_current</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Battery Pack B state of charge</t>
+          <t>Battery Pack B current (signed, +disch / -regen)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>System/CANBusSystem/cBMSB/SOC</t>
+          <t>System/CANBusSystem/cBMSB/Current</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0</v>
+        <v>-800</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>100</v>
+        <v>800</v>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>1 s</t>
+          <t>250 ms</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Pack B energy level; LOAD-010</t>
+          <t>High speed Pack B current; PERF-008</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1562,90 +1562,182 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>bmsb_soc</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack B state of charge</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSB/SOC</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>1 s</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Pack B energy level; LOAD-010</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t>bmsb_temp_max</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Battery Pack B maximum cell temperature</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>System/CANBusSystem/cBMSB/MaxTemp</t>
         </is>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E24" s="5" t="n">
         <v>-20</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F24" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>5 s</t>
         </is>
       </c>
-      <c r="H23" s="7" t="n">
+      <c r="H24" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Pack B thermal monitoring</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>present</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>bmsb_soh</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Battery Pack B State of Health</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>System/CANBusSystem/cBMSB/SOH</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>1.16e-05</v>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Metric1d</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>ambient_temp</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Ambient temperature</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E26" s="10" t="n">
         <v>-20</v>
       </c>
-      <c r="F24" s="10" t="n">
+      <c r="F26" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="G24" s="13" t="inlineStr">
+      <c r="G26" s="13" t="inlineStr">
         <is>
           <t>1 min</t>
         </is>
       </c>
-      <c r="H24" s="11" t="n">
+      <c r="H26" s="11" t="n">
         <v>0.0167</v>
       </c>
-      <c r="I24" s="9" t="inlineStr">
+      <c r="I26" s="9" t="inlineStr">
         <is>
           <t>Normalise performance results</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>manual-only</t>
         </is>

</xml_diff>